<commit_message>
criação de robo APPA
</commit_message>
<xml_diff>
--- a/cronograma_GEMAQ_30_12_2025.xlsx
+++ b/cronograma_GEMAQ_30_12_2025.xlsx
@@ -38,12 +38,18 @@
       <sz val="8"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D3D3D3"/>
+        <bgColor rgb="00D3D3D3"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -53,8 +59,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D3D3D3"/>
-        <bgColor rgb="00D3D3D3"/>
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
     <fill>
@@ -82,7 +88,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -90,13 +96,16 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -464,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -515,347 +524,443 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>006/2025</t>
+          <t>21 | Processo 142/2025</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Credenciamento</t>
+          <t>Dispensa</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE AMARGOSA</t>
+          <t>MUNICIPIO DE ALTO PARAISO</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>CREDENCIAMENTO DE EMPRESAS E/OU PROFISSIONAIS PARA A PRESTAÇÃO DE SERVIÇOS DEMANUTENÇÃO DE TRATORES, RETROESCAVADEIRAS, PATROL E MAQUINÁRIO AFIM PERTENCENTES À FROTA DOMUNICÍPIO DE AMARGOSA/BA.</t>
+          <t>CONTRATACAO DE EMPRESA ESPECIALIZADA PARA A LOCACAO DE BRINQUEDOS E PRESTACAO DE SERVICOS RECREATIVOS DESTINADOS A REALIZACAO DE DIVERSOS EVENTOS PROMOVIDOS PELA SECRETARIA MUNICIPAL DE PROMOCAO SOCIAL DE ALTO PARAISO   PR  INCLUINDO  ENTRE OUTROS  LOCACAO DE BRINQUEDOS INFLAVEIS  OFICINAS DE PULSEI</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>983319</t>
+          <t>0000</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>31/12/2025 08:30</t>
+          <t>31/12/2025 12:00</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>004/2025</t>
+          <t>23/2025</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Dispensa</t>
+          <t>Credenciamento</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>CONSORCIO DE DESENVOLVIMENTO SUSTENTAVEL DO TERRITORIO PIEMONTE NORTE DO ITAPICURU - CDS SENHOR DO BONFIM</t>
+          <t>CONSELHO REGIONAL DE CONTABILIDADE DO PARANA</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>DESTINA-SE À AQUISIÇÃO DE UMA BUCHA FLAGEADA E UMA BUCHA DE AÇO, PARA REPOSIÇÃO NA PATROL, LOTADO NA USINA ASFALTICA DO CDS. EM: 2/1/2025</t>
+          <t>CREDENCIAMENTO DE PESSOAS JURÍDICAS INTERESSADAS EM FIRMAR ACORDO DE PATROCÍNIO PARA APOIO DE EVENTOS ORGANIZADOS PELO CRCPR.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>925154</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>31/12/2025 14:00</t>
+          <t>31/12/2025 18:00</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>04/2025</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
+          <t>PRI 12/2025</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Credenciamento</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE SANTO ANTONIO DE JESUS</t>
+          <t>MUNICIPIO DE CORBELIA</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE MÃO-DE-OBRA ATRAVÉS DO CREDENCIAMENTO DE MICROEMPREENDEDORES INDIVIDUAIS (MEIS) E PESSOAS FÍSICAS PARA PRESTAÇÃO DOS SERVIDORES DE OPERADORES DE MOTONIVELADORA, PÁ CARREGADEIRA, RETROESCAVADEIRA, CAÇAMBAS E TRATORES, PARA ATENDER ÀS DEMANDAS DO MUNICÍPIO DE SANTO ANTÔNIO DE JESUS/BA</t>
+          <t>CONSTITUI OBJETO DO PRESENTE PROCESSO, O CREDENCIAMENTO DE EMPRESAS ESPECIALIZADAS PARA A PRESTAÇÃO DE SERVIÇOS COMO PROFESSOR DE EDUCAÇÃO FÍSICA, GRADUADO E COM BACHARELADO, COM REGISTRO NO CONSELHO REGIONAL DE EDUCAÇÃO FÍSICA - CREF/PR E CONSELHO FEDERAL DE EDUCAÇÃO FÍSICA - CONFEF, PARA ATUAR NA SECRETARIA MUNICIPAL DE ESPORTES E LAZER EM TREINAMENTOS ESPORTIVOS E EM EVENTOS REALIZADOS NO MUNICÍPIO DE CORBÉLIA/PR.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>1865</t>
+          <t>09002</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>31/12/2025 23:59</t>
+          <t>31/12/2025 18:00</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>CD Nº 004/2025/2025</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
+          <t>2/2025</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Credenciamento</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE CASTRO ALVES</t>
+          <t>UNIVERSIDADE ESTADUAL DE LONDRINA</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE PESSOA FÍSICA/JURÍDICA PARA PRESTAÇÃO DE SERVIÇO DE LOCAÇÃO DE EQUIPAMENTO TIPO TRATOR AGRÍCOLA, VISANDO REALIZAR A ARAÇÃO COMUNITÁRIA, PARA ATENDIMENTO DOS AGRICULTORES FAMILIARES DO MUNICÍPIO DE CASTRO ALVES</t>
+          <t>CHAMAMENTO PUBLICO N. 04/2024 - CREDENCIAMENTO DE RESTAURANTES PARA FORNECIMENTO DE SERVIÇOS DEALIMENTAÇÃO (ALMOÇO E/OU JANTAR) VISANDO O ATENDIMENTO DE PALESTRANTESCONVIDADOS EM EVENTOS PROMOVIDOS PELA UEL/PROEX E/OU DOCENTES CONVIDADOSPARA MINISTRAR AULAS NOS PROGRAMAS DE PÓS-GRADUAÇÃO (UEL/PROPPG), BEM COMOATENDER OUTRAS UNIDADES INSTITUIÇÃO QUE NECESSITEM DOS SERVIÇOS</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2101</t>
+          <t>926769</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>06/01/2026 08:00</t>
+          <t>31/12/2025 18:00</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>016/2025</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Pregão - Eletrônico</t>
+          <t>6/2026</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Credenciamento</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>CONSORCIO DE DESENVOLVIMENTO SUSTENTAVEL DO VALE DO JIQUIRICA - CDSVJ</t>
+          <t>UNIVERSIDADE ESTADUAL DE LONDRINA</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>PREGÃO ELETRÔNICO SRP PARA FUTURA  E EVENTUAL CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NO FORNECIMENTO DE 01 (UMA)  RETROESCAVADEIRA HIDRÁULICA, PARA ATENDER ÀS NECESSIDADES DO CONVALE, TUDO CONFORME CRITÉRIOS ESTABELECIDOS NO EDITAL E TERMO DE REFERÊNCIA.</t>
+          <t>CREDENCIAMENTO DE RESTAURANTES PARA FORNECIMENTO DE SERVIÇOS DE ALIMENTAÇÃO (ALMOÇO E/OU JANTAR) VISANDO O ATENDIMENTO DE PALESTRANTES CONVIDADOS EM EVENTOS PROMOVIDOS PELA UEL/PROEX E/OU DOCENTES CONVIDADOS PARA MINISTRAR AULAS NOS PROGRAMAS DE PÓS-GRADUAÇÃO (UEL/PROPPG), BEM COMO ATENDER OUTRAS UNIDADES INSTITUIÇÃO QUE NECESSITEM DOS SERVIÇOS.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>000000001</t>
+          <t>926769</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>06/01/2026 08:30</t>
+          <t>05/01/2026 09:00</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>PE043/2025</t>
+          <t>23/2025</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Pregão - Eletrônico</t>
+          <t>Pregão - Presencial</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE IBIRAPITANGA</t>
+          <t>MUNICIPIO DE NOVA OLIMPIA</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>REGISTRO DE PREÇOS PARA FUTURA E EVENTUAL AQUISIÇÃO DE MÁQUINAS PESADAS, TIPO MOTONIVELADORA, PÁ CARREGADEIRA, RETROESCAVADEIRA E ROLO COMPACTADOR, DESTINADAS AO FORTALECIMENTO DAS AÇÕES DE INFRAESTRUTURA URBANA E RURAL DO MUNICÍPIO DE IBIRAPITANGA-BA.</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA A PRESTAÇÃO DE SERVIÇOS DE DECORAÇÃO E ORNAMENTAÇÃO, COM LOCAÇÃO DE ITENS DECORATIVOS E AQUISIÇÃO DE MATERIAIS DE CONSUMO DESTINADOS AOS EVENTOS, COMEMORAÇÕES E À MONTAGEM DE LEMBRANÇAS PROMOVIDOS PELO MUNICÍPIO DE NOVA OLÍMPIA/PR.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>000000001</t>
+          <t>75799577000104</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>07/01/2026 08:00</t>
+          <t>05/01/2026 09:00</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>020/2025</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
+          <t>90007/2025</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Pregão - Eletrônico</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE CATURAMA</t>
+          <t>CAMARA MUNICIPAL DE CAMBE</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AQUISIÇÃO DE MÁQUINA (TRATOR) PARA ATENDER ÀS DEMANDAS DO MUNICÍPIO DE CATURAMA-BA, CONFORME CONVÊNIO TRASNFEREGOV Nº 982151/2025 E AS CONDIÇÕES ESTABELECIDAS EM EDITAL E SEUS ANEXOS. </t>
+          <t>AQUISIÇÃO DE EQUIPAMENTOS, SOFTWARES E ACESSÓRIOS DE ÁUDIO, VÍDEO, INFORMÁTICA E REDE, DESTINADOS À CAPTAÇÃO, PRODUÇÃO, CONTROLE E TRANSMISSÃO DAS SESSÕES LEGISLATIVAS E EVENTOS INSTITUCIONAIS DA CÂMARA MUNICIPAL DE CAMBÉ/PR, CONFORME ESPECIFICAÇÕES, QUANTITATIVOS E CONDIÇÕES ESTABELECIDOS NO TERMO DE REFERÊNCIA.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>000000001</t>
+          <t>927678</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>12/01/2026 00:00</t>
+          <t>06/01/2026 08:29</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>051/2025</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
+          <t>90123/2025</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>Pregão - Eletrônico</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE RIBEIRA DO AMPARO</t>
+          <t>MUNICIPIO DE CANDOI</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA PARA AQUISIÇÃO DE MÁQUINAS (RETROESCAVADEIRA) DESTINADA AS DEMANDAS DA SECRETARIA MUNICIPAL DE AGRICULTURA CONFORME CONVÊNIO TRANSFEREGOV.BR Nº 986597/2025 CELEBRADO, ENTRE A UNIÃO, POR INTERMÉDIO DO MINISTÉRIO DA INTEGRAÇÃO E DO DESENVOLVIMENTO REGIONAL, E O MUNICÍPIO DE RIBEIRA DO AMPARO/BA</t>
+          <t>REGISTRO DE PREÇOS DE GÊNEROS ALIMENTÍCIOS, SORVETES, PICOLÉS E CHOCOLATES, DESTINADOS À MERENDA ESCOLAR, ALIMENTAÇÃO DOS BOMBEIROS, DOS INSTITUCIONALIZADOS NA CASAR LAR, DA BANDA MUNICIPAL E ATLETAS QUANDO ESTIVEREM EM VIAGENS REPRESENTANDO O MUNICÍPIO, E PARA CONSUMO EM PROGRAMAS SOCIAIS, REUNIÕES, PALESTRAS E DEMAIS EVENTOS PÚBLICOS MUNICIPAIS</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>12/01/2026 09:00</t>
+          <t>06/01/2026 09:28</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>90032/2025</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
+          <t>PE 90/2025</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Pregão - Eletrônico</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE MARAGOGIPE</t>
+          <t>MUNICIPIO DE CORNELIO PROCOPIO</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA A PRESTAÇÃO DE SERVIÇOS DE LIMPEZA DE RUAS COM VARRIÇÃO, ROÇAGEM, CAPINA, PINTURA DE MEIO FIO, PODA DE ÁRVORES, DESASSOREAMENTO DE CANAIS E CÓRREGOS, ROÇAGEM MECANIZADA COM TRATOR, E RETIRADA E TRANSPORTE DE RESÍDUOS E ENTULHOS, COM FORNECIMENTO DE TODOS OS MATERIAIS, EQUIPAMENTOS, VEÍCULOS E MÁQUINAS NECESSÁRIOS PARA A EXECUÇÃO DOS SERVIÇOS, EM ATENDIMENTO AS DEMANDAS DO MUNICÍPIO DE MARAGOJIPE-BA.</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA O FORNECIMENTO DE TRIO ELÉTRICO COMPLETO, INCLUINDO TODA A ESTRUTURA TÉCNICA, SOM, ILUMINAÇÃO, PAINEL DE LED, EQUIPE TÉCNICA E LOGÍSTICA OPERACIONAL, PARA A REALIZAÇÃO DOS EVENTOS CARNAVALESCOS DO MUNICÍPIO DE CORNÉLIO PROCÓPIO/PR, NO PERÍODO DE 13 A 16 DE FEVEREIRO DE 2026</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>983713</t>
+          <t>4582</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>12/01/2026 10:00</t>
+          <t>09/01/2026 23:59</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>051/2025</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Pregão - Eletrônico</t>
+          <t>PRI 182/2025</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Credenciamento</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE RIBEIRA DO AMPARO</t>
+          <t>MUNICIPIO DE CAMPO MOURAO</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>[LICITANET] - CONTRATAÇÃO DE EMPRESA PARA AQUISIÇÃO DE MÁQUINAS (RETROESCAVADEIRA) DESTINADA AS DEMANDAS DA SECRETARIA MUNICIPAL DE AGRICULTURA CONFORME CONVÊNIO TRANSFEREGOV.BR Nº 986597/2025 CELEBRADO, ENTRE A UNIÃO, POR INTERMÉDIO DO MINISTÉRIO DA INTEGRAÇÃO E DO DESENVOLVIMENTO REGIONAL, E O MUNICÍPIO DE RIBEIRA DO AMPARO/BA</t>
+          <t>CHAMAMENTO PÚBLICO, COM O OBJETIVO DE FORMALIZAR PARCERIA, POR MEIO DE TERMO DE COLABORAÇÃO COM ORGANIZAÇÃO DA SOCIEDADE CIVIL (OSC), VISANDO À VINCULAÇÃO JUNTO AO COMITÊ BRASILEIRO DE CLUBES - CBC PARA VIABILIZAÇÃO DA PARTICIPAÇÃO DE ATLETAS QUE REPRESENTAM O MUNICÍPIO EM COMPETIÇÕES E/OU EVENTOS ESPORTIVOS</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>3057</t>
+          <t>03001</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>13/01/2026 07:00</t>
+          <t>12/01/2026 08:00</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>067/2025 PE/2025</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
+          <t>48/2025</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>Pregão - Eletrônico</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE SANTO ESTEVAO</t>
+          <t>MUNICIPIO DE GUAMIRANGA</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA PRESTAÇÃO DE SERVIÇO DE LOCAÇÃO DE HORA/MÁQUINA (TRATOR AGRÍCOLA), EQUIPADO COM ARADO DE DISCOS, INCLUINDO OPERADOR, COMBUSTÍVEL E MANUTENÇÃO, VISANDO ATENDER ÀS NECESSIDADES DA SECRETARIA MUNICIPAL DE AGRICULTURA, PECUÁRIA, DESENVOLVIMENTO ECONÔMICO E </t>
+          <t xml:space="preserve">ESTA ATA DE REGISTRO DE PREÇO PARA O FORNECIMENTO, FUTURO E PARCELADO DE MATERIAIS DE CONSUMO (GÊNEROS ALIMENTÍCIOS E MERCADORIAS), PARA USO DA SECRETARIA DE AGRICULTURA, PECUÁRIA E MEIO AMBIENTE PARA REALIZAÇÃO DOS CURSOS, REUNIÕES E EVENTOS PARA OS PRODUTORES RURAIS, PELO PERÍODO DE 12 (DOZE) MESES, CONFORME ESPECIFICAÇÕES, QUANTIDADES E CONDIÇÕES ESTABELECIDAS NO TERMO DE REFERÊNCIA E NESTE EDITAL. </t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
           <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>13/01/2026 08:00</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>PCE 82/2025</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Pregão - Eletrônico</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>MUNICIPIO DE COLOMBO</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>CONTRATAÇÃO DE EMPRESA PARA PRESTAÇÃO DE SERVIÇOS EM LOCAÇÃO DE ESTRUTURAS DE EVENTOS PARA ATUAR NA 59ª FESTA DA UVA NO MUNICÍPIO DE COLOMBO/PR, COMPREENDENDO AS QUANTIDADES E ESPECIFICAÇÕES E, CONFORME CONDIÇÕES E EXIGÊNCIAS ESTABELECIDAS NO TERMO DE REFERÊNCIA</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>21002</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>13/01/2026 08:28</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>PE 94/2025</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Pregão - Eletrônico</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>MUNICIPIO DE CORNELIO PROCOPIO</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS CONTÍNUOS DE SEGURANÇA PRIVADA DESARMADA, SOB O REGIME DE DEDICAÇÃO EXCLUSIVA DE MÃO DE OBRA SOMENTE EM HORÁRIOS EFETIVAMENTE CONVOCADO PELA ADMINISTRAÇÃO, MEDIDOS POR HORA-SEGURANÇA (HS), PARA ATENDER ÀS DEMANDAS DE SEGURANÇA DAS FESTIVIDADES, EVENTOS CULTURAIS, ESPORTIVOS E INSTITUCIONAIS PROMOVIDOS PELO MUNICÍPIO.</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>4582</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>13/01/2026 08:59</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>PCE 184/2025</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Pregão - Eletrônico</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>MUNICIPIO DE CASCAVEL</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>ADQUIRIR DOIS ÔNIBUS PARA A SECRETARIA MUNICIPAL DE ESPORTE E LAZER GARANTIR O TRANSPORTE SEGURO, EFICIENTE E ADEQUADO DE ATLETAS, EQUIPES TÉCNICAS E PARTICIPANTES DE EVENTOS ESPORTIVOS REPRESENTANDO O MUNICÍPIO EM COMPETIÇÕES, TORNEIOS, JOGOS E ATIVIDADES RECREATIVAS DENTRO E FORA DA CIDADE.</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>37001</t>
         </is>
       </c>
     </row>

</xml_diff>